<commit_message>
Add .gitignore to block large datasets and models
</commit_message>
<xml_diff>
--- a/results/training.xlsx
+++ b/results/training.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\projects\RF_DCOPF\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03FD2C41-BB96-4787-856F-6FC38E0700C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDB1355B-B598-4226-BE3B-CE5D2238A46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="85">
   <si>
     <t>pglib_opf_case73_ieee_rts</t>
   </si>
@@ -91,19 +91,220 @@
   </si>
   <si>
     <t>8.82% ± 0.66%</t>
+  </si>
+  <si>
+    <t>83.20% ± 0.36%</t>
+  </si>
+  <si>
+    <t>75.78% ± 1.09%</t>
+  </si>
+  <si>
+    <t>72.96% ± 0.94%</t>
+  </si>
+  <si>
+    <t>90.66% ± 0.89%</t>
+  </si>
+  <si>
+    <t>82.92% ± 0.62%</t>
+  </si>
+  <si>
+    <t>78.58% ± 0.93%</t>
+  </si>
+  <si>
+    <t>66.62% ± 1.19%</t>
+  </si>
+  <si>
+    <t>33.48% ± 1.22%</t>
+  </si>
+  <si>
+    <t>11.22% ± 0.59%</t>
+  </si>
+  <si>
+    <t>51.64% ± 1.11%</t>
+  </si>
+  <si>
+    <t>29.20% ± 0.36%</t>
+  </si>
+  <si>
+    <t>13.14% ± 0.88%</t>
+  </si>
+  <si>
+    <t>89.80% ± 0.53%</t>
+  </si>
+  <si>
+    <t>83.72% ± 0.63%</t>
+  </si>
+  <si>
+    <t>80.50% ± 1.05%</t>
+  </si>
+  <si>
+    <t>84.92% ± 0.54%</t>
+  </si>
+  <si>
+    <t>80.74% ± 0.27%</t>
+  </si>
+  <si>
+    <t>77.58% ± 1.85%</t>
+  </si>
+  <si>
+    <t>97.32% ± 0.41%</t>
+  </si>
+  <si>
+    <t>89.26% ± 0.48%</t>
+  </si>
+  <si>
+    <t>75.24% ± 1.13%</t>
+  </si>
+  <si>
+    <t>77.02% ± 1.15%</t>
+  </si>
+  <si>
+    <t>68.98% ± 1.13%</t>
+  </si>
+  <si>
+    <t>42.32% ± 1.32%</t>
+  </si>
+  <si>
+    <t>98.66% ± 0.26%</t>
+  </si>
+  <si>
+    <t>93.18% ± 0.34%</t>
+  </si>
+  <si>
+    <t>83.60% ± 1.10%</t>
+  </si>
+  <si>
+    <t>81.22% ± 0.97%</t>
+  </si>
+  <si>
+    <t>77.38% ± 0.63%</t>
+  </si>
+  <si>
+    <t>99.76% ± 0.15%</t>
+  </si>
+  <si>
+    <t>96.04% ± 0.39%</t>
+  </si>
+  <si>
+    <t>93.48% ± 0.94%</t>
+  </si>
+  <si>
+    <t>74.26% ± 0.83%</t>
+  </si>
+  <si>
+    <t>50.92% ± 1.63%</t>
+  </si>
+  <si>
+    <t>90.52% ± 0.38%</t>
+  </si>
+  <si>
+    <t>77.96% ± 0.92%</t>
+  </si>
+  <si>
+    <t>92.80% ± 0.32%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">88.80% ± 0.33% </t>
+  </si>
+  <si>
+    <t>85.96% ± 1.55%</t>
+  </si>
+  <si>
+    <t>83.42% ± 0.55%</t>
+  </si>
+  <si>
+    <t>60.50% ± 1.01%</t>
+  </si>
+  <si>
+    <t>49.82% ± 0.89%</t>
+  </si>
+  <si>
+    <t>72.22% ± 0.70%</t>
+  </si>
+  <si>
+    <t>83.44% ± 0.67%</t>
+  </si>
+  <si>
+    <t>96.26% ± 0.45%</t>
+  </si>
+  <si>
+    <t>72.36% ± 1.24%</t>
+  </si>
+  <si>
+    <t>66.78% ± 1.12%</t>
+  </si>
+  <si>
+    <t>48.26% ± 0.51%</t>
+  </si>
+  <si>
+    <t>99.86% ± 0.08%</t>
+  </si>
+  <si>
+    <t>97.64% ± 0.26%</t>
+  </si>
+  <si>
+    <t>95.52% ± 0.27%</t>
+  </si>
+  <si>
+    <t>100.00% ± 0.00%</t>
+  </si>
+  <si>
+    <t>46.04% ± 2.12%</t>
+  </si>
+  <si>
+    <t>3.24% ± 0.42%</t>
+  </si>
+  <si>
+    <t>0.12% ± 0.07%</t>
+  </si>
+  <si>
+    <t>99.26% ± 0.08%</t>
+  </si>
+  <si>
+    <t>71.08% ± 0.48%</t>
+  </si>
+  <si>
+    <t>42.64% ± 0.98%</t>
+  </si>
+  <si>
+    <t>97.14% ± 0.52%</t>
+  </si>
+  <si>
+    <t>82.04% ± 0.68%</t>
+  </si>
+  <si>
+    <t>40.54% ± 1.38%</t>
+  </si>
+  <si>
+    <t>23.40% ± 0.61%</t>
+  </si>
+  <si>
+    <t>10.88% ± 1.09%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF202020"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -126,9 +327,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -414,29 +617,32 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="B1" s="2">
+      <c r="B1" s="4">
         <v>0.01</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2">
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4">
         <v>0.03</v>
       </c>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2">
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4">
         <v>0.5</v>
       </c>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
@@ -495,67 +701,265 @@
       <c r="C3" t="s">
         <v>16</v>
       </c>
+      <c r="D3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="G3" t="s">
         <v>20</v>
       </c>
       <c r="H3" t="s">
         <v>17</v>
       </c>
+      <c r="I3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="L3" t="s">
         <v>21</v>
       </c>
       <c r="M3" t="s">
         <v>18</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
+      <c r="B4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2</v>
       </c>
+      <c r="B5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
+      <c r="B6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
+      <c r="B7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="O7" s="3" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
+      <c r="B8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
+      <c r="E9" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>6</v>
       </c>
+      <c r="E10" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>7</v>
       </c>
+      <c r="E11" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
+      <c r="E12" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="O13" s="3" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -565,5 +969,6 @@
     <mergeCell ref="L1:P1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>